<commit_message>
Changes to steps.py and test_quote_fg_ho_wind.py to add foundation elevation field if visible. Also, renamed test_fg_ho_wind_v2.py to test_v2fg_ho_wind_.py
</commit_message>
<xml_diff>
--- a/fg_test_results.xlsx
+++ b/fg_test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,12 +456,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9607 Bahia Rd, Ocala, FL 34472</t>
+          <t>15110 Shearcrest Dr, Lithia, FL 33547</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>HO-3</t>
+          <t>HO Wind Only</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>QD20045309</t>
+          <t>QD20045356</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>$7,904.30</t>
+          <t>$3,175.20</t>
         </is>
       </c>
     </row>
@@ -488,12 +488,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7733 Belvoir Dr, Orlando, FL 32835</t>
+          <t>612 Citrus Wood Ln, Valrico, FL 33594</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HO-3 Tenant</t>
+          <t>HO Wind Only</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -503,12 +503,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>QD20045310</t>
+          <t>QD20045358</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>$5,708.75</t>
+          <t>$3,597.30</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8734 Crestgate Cir, Orlando, FL 32819</t>
+          <t>12274 Accipiter Dr, Orlando, FL 32837</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -535,76 +535,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>QD20045311</t>
+          <t>QD20045359</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>$8,447.25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>tsicortesmarquez@geovera</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>3319 Clubview Dr, North Fort Myers, FL 33917</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Basic Form</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>QD20045312</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>$9,146.45</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>tsicortesmarquez@geovera</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>3408 69th St W, Lehigh Acres, FL 33971</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Broad Form</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>QD20045313</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>$3,179.30</t>
+          <t>$3,824.10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing updates to hl tests
</commit_message>
<xml_diff>
--- a/fg_test_results.xlsx
+++ b/fg_test_results.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,8 +412,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="36" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="51.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="16" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="14.42578125" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -541,6 +547,198 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>$3,824.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8832 Savona Ct, Naples, FL 34119</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HO-3 Tenant</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>800,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>QD20045360</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>$4,493.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8832 Savona Ct, Naples, FL 34119</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HO Wind Only</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>800,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>QD20045361</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>$3,920.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3419 26th St SW, Lehigh Acres, FL 33976</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Short-Term Vacant or Unoccupied Dwelling - Basic Form</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>600,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>QD20045362</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>$2,527.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>612 Citrus Wood Ln, Valrico, FL 33594</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HO Wind Only</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>800,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>QD20045364</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>$3,597.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>9426 Meadow Crest Ln, Clermont, FL 34711</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>HO-3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>800,000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>QD20045365</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>$4,675.55</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tsicortesmarquez@geovera</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3618 Elm St, Ellenton, FL 34222</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Short-Term Vacant or Unoccupied Dwelling - Broad Form</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>600,000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>QD20045366</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>$3,365.15</t>
         </is>
       </c>
     </row>

</xml_diff>